<commit_message>
SORT_DATA 자동 동기화: Answersheet 신규 리뷰 추가 (#30, 4CE Dimension)
검색어_맵핑.xlsx에 Answersheet 행 추가 (키워드는 비어둠)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1000,26 +1000,21 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Answersheet</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1029,12 +1024,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>키이스케이프</t>
+          <t>tumbleweed</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>keyescape</t>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1041,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1063,12 +1058,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1075,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>구스리아</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1097,12 +1092,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>ぐずりあ</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1114,12 +1109,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
         </is>
       </c>
     </row>
@@ -1131,29 +1126,29 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1164,6 +1159,23 @@
         </is>
       </c>
       <c r="B41" t="inlineStr">
+        <is>
+          <t>SCRAP - Mystery For You</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>4CE Dimension</t>
         </is>

</xml_diff>

<commit_message>
SORT_DATA 자동 동기화: ECO 신규 리뷰 추가 (#31, Tumbleweed)
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1012,26 +1012,21 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ECO</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1041,12 +1036,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>키이스케이프</t>
+          <t>tumbleweed</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>keyescape</t>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1058,12 +1053,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1070,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1092,12 +1087,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>구스리아</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1104,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>ぐずりあ</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1121,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
         </is>
       </c>
     </row>
@@ -1143,29 +1138,29 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1176,6 +1171,23 @@
         </is>
       </c>
       <c r="B42" t="inlineStr">
+        <is>
+          <t>SCRAP - Mystery For You</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>4CE Dimension</t>
         </is>

</xml_diff>

<commit_message>
sync 스크립트: 엑셀 키워드 자동 → PHONETIC_MAP/COMPANY_MAP 반영
- read_xlsx_keywords/apply_xlsx_to_maps 추가
- 미반영 8건 일괄 적용 (AXIDENTZ, タンブルダイス, はじみまして,
  Answersheet, ECO, アナビナゾ, 4CE Dimension, AnotherVision)
- 검색어_맵핑.xlsx: アルティメットナゾトキショウ 부가 표기 제거
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/monbbang/Library/Mobile Documents/com~apple~CloudDocs/MacBook Air M2/나조토키/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4376728C-DE45-7F4A-8A28-ED749C6A2733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA3F71F-58F3-F34C-B418-B388ED472D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,9 +88,6 @@
     <t>히라메키 트럼프 실버, 히라메키트럼프 실버, 히라메키트럼프실버, 히라메키 트럼프실버, 히라메키, 트럼프, 실버</t>
   </si>
   <si>
-    <t>アルティメットナゾトキショウ (얼티밋 나조토키쇼)</t>
-  </si>
-  <si>
     <t>얼티밋 나조토키쇼, 얼티밋나조토키쇼, 궁극의 나조토키쇼, 궁극의나조토키쇼, 얼티밋, 나조토키, 쇼</t>
   </si>
   <si>
@@ -295,6 +292,10 @@
   </si>
   <si>
     <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>アルティメットナゾトキショウ</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -406,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -417,7 +418,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -842,11 +842,11 @@
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -854,10 +854,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -865,10 +865,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -876,10 +876,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -887,10 +887,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -898,10 +898,10 @@
         <v>3</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -909,10 +909,10 @@
         <v>3</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -920,10 +920,10 @@
         <v>3</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -931,10 +931,10 @@
         <v>3</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -942,10 +942,10 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -953,10 +953,10 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -964,10 +964,10 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -975,10 +975,10 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -986,10 +986,10 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -997,10 +997,10 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1008,10 +1008,10 @@
         <v>3</v>
       </c>
       <c r="B26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1019,10 +1019,10 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1030,10 +1030,10 @@
         <v>3</v>
       </c>
       <c r="B28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1041,10 +1041,10 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1052,10 +1052,10 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>60</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1063,10 +1063,10 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1074,10 +1074,10 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>88</v>
+        <v>63</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1085,10 +1085,10 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>89</v>
+        <v>64</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1098,123 +1098,123 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>79</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C42" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B43" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B44" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B45" t="s">
-        <v>87</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SORT_DATA 자동 동기화: 馬崎 春のぱずる祭り 2026 신규 리뷰 추가 (#34, SCRAP - Mystery For You)
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1078,26 +1078,21 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>馬崎 春のぱずる祭り 2026</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1107,12 +1102,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>키이스케이프</t>
+          <t>tumbleweed</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>keyescape</t>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1124,12 +1119,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1136,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1153,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>구스리아</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1170,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>ぐずりあ</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1187,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
         </is>
       </c>
     </row>
@@ -1209,29 +1204,29 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1238,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>4CE Dimension</t>
+          <t>SCRAP - Mystery For You</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>포스 디멘션, 포스 디멘젼</t>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1260,10 +1255,27 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>4CE Dimension</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>포스 디멘션, 포스 디멘젼</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>AnotherVision</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
         </is>

</xml_diff>

<commit_message>
SORT_DATA 자동 동기화: FouRe, Collection : lie, 馬崎 春のぱずる祭り2026 신규 리뷰 추가 (#36~#38, SCRAP - Mystery For You)
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1113,60 +1113,45 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>FouRe:</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Collection : lie</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>키이스케이프</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>keyescape</t>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>馬崎 春のぱずる祭り2026</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1176,12 +1161,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>tumbleweed</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1193,12 +1178,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>구스리아</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1210,12 +1195,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1227,12 +1212,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>MICHI</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1244,61 +1229,112 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
+          <t>ぐずりあ</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>구스리아</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>SCRAP - Mystery For You</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C49" s="8" t="inlineStr">
         <is>
           <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>4CE Dimension</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t>포스 디멘션, 포스 디멘젼</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>AnotherVision</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
         </is>

</xml_diff>

<commit_message>
SORT_DATA 자동 동기화: パズバコ 신규 리뷰 추가 (#39, SCRAP), FouRe puzzle 3.9→3.8
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1149,26 +1149,21 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>パズバコ</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
-        </is>
-      </c>
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1178,12 +1173,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>키이스케이프</t>
+          <t>tumbleweed</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>keyescape</t>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1195,12 +1190,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1212,12 +1207,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1224,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>구스리아</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1246,12 +1241,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>ぐずりあ</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1263,12 +1258,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
         </is>
       </c>
     </row>
@@ -1280,29 +1275,29 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1309,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>4CE Dimension</t>
+          <t>SCRAP - Mystery For You</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>포스 디멘션, 포스 디멘젼</t>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1331,10 +1326,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>4CE Dimension</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>포스 디멘션, 포스 디멘젼</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>AnotherVision</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
         </is>

</xml_diff>

<commit_message>
리뷰 #58 HIRAMEKI TRUMP RED, #59 HIRAMEKI TRUMP 추가
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XtnWGBiPRWjUEmzryHdoz
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1293,43 +1293,33 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HIRAMEKI TRUMP RED</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HIRAMEKI TRUMP</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>키이스케이프</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>keyescape</t>
-        </is>
-      </c>
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1339,12 +1329,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>tumbleweed</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1356,12 +1346,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1373,12 +1363,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>구스리아</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1390,12 +1380,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1407,12 +1397,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>ぐずりあ</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1424,46 +1414,46 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>4CE Dimension</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>포스 디멘션, 포스 디멘젼</t>
         </is>
       </c>
     </row>
@@ -1475,12 +1465,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>AnotherVision</t>
+          <t>SCRAP - Mystery For You</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1482,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>xeoxy</t>
+          <t>4CE Dimension</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>포스 디멘션, 포스 디멘젼</t>
         </is>
       </c>
     </row>
@@ -1503,6 +1498,35 @@
         </is>
       </c>
       <c r="B65" t="inlineStr">
+        <is>
+          <t>AnotherVision</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>xeoxy</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>リドラ</t>
         </is>

</xml_diff>

<commit_message>
검색어 맵핑: Premium One vol.1 -THE CARDS- 행 추가 (b06f50c 누락분)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1562,26 +1562,21 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Premium One vol.1 -THE CARDS-</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
-        </is>
-      </c>
+      <c r="A64" s="2" t="n"/>
+      <c r="B64" s="2" t="n"/>
+      <c r="C64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1591,12 +1586,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>키이스케이프</t>
+          <t>tumbleweed</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>keyescape</t>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1608,12 +1603,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1625,12 +1620,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1637,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>구스리아</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1654,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>ぐずりあ</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1671,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
         </is>
       </c>
     </row>
@@ -1693,29 +1688,29 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1722,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>4CE Dimension</t>
+          <t>SCRAP - Mystery For You</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>포스 디멘션, 포스 디멘젼</t>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1744,12 +1739,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>AnotherVision</t>
+          <t>4CE Dimension</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
+          <t>포스 디멘션, 포스 디멘젼</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1756,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>xeoxy</t>
+          <t>AnotherVision</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>제옥시</t>
+          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
         </is>
       </c>
     </row>
@@ -1778,12 +1773,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>リドラ</t>
+          <t>xeoxy</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>리도라, 리들러</t>
+          <t>제옥시</t>
         </is>
       </c>
     </row>
@@ -1795,29 +1790,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ねずみの巣</t>
+          <t>リドラ</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>쥐의굴, 쥐의 굴, 네즈미노 스, 쥐의둥지, 쥐의 둥지, 쥐의 보금자리, 쥐의보금자리, 쥐집, 쥐 집, 쥐의집, 쥐의 집</t>
+          <t>리도라, 리들러</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>나조 이름</t>
+          <t>브랜드</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>HIRAMEKI TRUMP</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>히라메키 트럼프, 히라메키트럼프, 히라메키, 트럼프</t>
+          <t>ねずみの巣</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>쥐의굴, 쥐의 굴, 네즈미노 스, 쥐의둥지, 쥐의 둥지, 쥐의 보금자리, 쥐의보금자리, 쥐집, 쥐 집, 쥐의집, 쥐의 집</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1824,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>HIRAMEKI TRUMP RED</t>
+          <t>HIRAMEKI TRUMP</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>히라메키 트럼프 레드, 히라메키트럼프 레드, 히라메키트럼프레드, 히라메키 트럼프레드, 레드, 히라메키, 트럼프</t>
+          <t>히라메키 트럼프, 히라메키트럼프, 히라메키, 트럼프</t>
         </is>
       </c>
     </row>
@@ -1846,10 +1841,27 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
+          <t>HIRAMEKI TRUMP RED</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>히라메키 트럼프 레드, 히라메키트럼프 레드, 히라메키트럼프레드, 히라메키 트럼프레드, 레드, 히라메키, 트럼프</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>XI</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>일레븐, 엑스아이</t>
         </is>

</xml_diff>

<commit_message>
검색어 맵핑: Premium One vol.2 -THE NUMBERS- 외 3건 행 추가 (이전 동기화 누락분)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1574,77 +1574,57 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="2" t="n"/>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Premium One vol.2 -THE NUMBERS-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>解錠</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>키이스케이프</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>keyescape</t>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>サイフアーカイブ</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>TUMBLEWEED HITS</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
-        </is>
-      </c>
+      <c r="A68" s="2" t="n"/>
+      <c r="B68" s="2" t="n"/>
+      <c r="C68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1654,12 +1634,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>구스리아</t>
+          <t>tumbleweed</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1651,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1688,12 +1668,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
+          <t>NAZOxNAZO劇団</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1705,80 +1685,80 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
+          <t>MICHI</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>미치</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>ぐずりあ</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>구스리아</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>4CE Dimension</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>포스 디멘션, 포스 디멘젼</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>AnotherVision</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>xeoxy</t>
-        </is>
-      </c>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>제옥시</t>
         </is>
       </c>
     </row>
@@ -1790,12 +1770,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>リドラ</t>
+          <t>SCRAP - Mystery For You</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>리도라, 리들러</t>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1807,61 +1787,129 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ねずみの巣</t>
+          <t>4CE Dimension</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>쥐의굴, 쥐의 굴, 네즈미노 스, 쥐의둥지, 쥐의 둥지, 쥐의 보금자리, 쥐의보금자리, 쥐집, 쥐 집, 쥐의집, 쥐의 집</t>
+          <t>포스 디멘션, 포스 디멘젼</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>나조 이름</t>
+          <t>브랜드</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>HIRAMEKI TRUMP</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>히라메키 트럼프, 히라메키트럼프, 히라메키, 트럼프</t>
+          <t>AnotherVision</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>나조 이름</t>
+          <t>브랜드</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>HIRAMEKI TRUMP RED</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>히라메키 트럼프 레드, 히라메키트럼프 레드, 히라메키트럼프레드, 히라메키 트럼프레드, 레드, 히라메키, 트럼프</t>
+          <t>xeoxy</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>제옥시</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>나조 이름</t>
+          <t>브랜드</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>リドラ</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>리도라, 리들러</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ねずみの巣</t>
+        </is>
+      </c>
+      <c r="C82" s="8" t="inlineStr">
+        <is>
+          <t>쥐의굴, 쥐의 굴, 네즈미노 스, 쥐의둥지, 쥐의 둥지, 쥐의 보금자리, 쥐의보금자리, 쥐집, 쥐 집, 쥐의집, 쥐의 집</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HIRAMEKI TRUMP</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>히라메키 트럼프, 히라메키트럼프, 히라메키, 트럼프</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>HIRAMEKI TRUMP RED</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>히라메키 트럼프 레드, 히라메키트럼프 레드, 히라메키트럼프레드, 히라메키 트럼프레드, 레드, 히라메키, 트럼프</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
           <t>XI</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>일레븐, 엑스아이</t>
         </is>

</xml_diff>